<commit_message>
fix: preserve spreadsheet and slide layout and speed offline preparation
</commit_message>
<xml_diff>
--- a/tests/fixtures/formatting.xlsx
+++ b/tests/fixtures/formatting.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <r>
       <t xml:space="preserve">Normal </t>
@@ -44,11 +44,34 @@
       <t>2</t>
     </r>
   </si>
+  <si>
+    <t>Percentage</t>
+  </si>
+  <si>
+    <t>HIDDEN</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Leading zeros</t>
+  </si>
+  <si>
+    <t>Fraction</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="0000"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -78,8 +101,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -419,12 +447,60 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="9" hidden="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1234.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="5">
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>